<commit_message>
Rename test client AA -> Client 1 (id C001) in template
https://claude.ai/code/session_013Pp3LR5u3aQiAWfkdUTFGV
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -439,10 +439,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AA</v>
+        <v>C001</v>
       </c>
       <c r="B2" t="str">
-        <v>Client AA</v>
+        <v>Client 1</v>
       </c>
       <c r="C2" t="str">
         <v>16:30</v>

</xml_diff>